<commit_message>
Stage 1 completion: video preprocessing, quality checks, DLC inference setup and trajectory analysis
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
@@ -573,7 +573,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
@@ -616,7 +616,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
@@ -659,7 +659,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
@@ -702,7 +702,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
@@ -745,7 +745,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
@@ -831,7 +831,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
@@ -874,7 +874,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -917,7 +917,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
@@ -960,7 +960,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">

</xml_diff>